<commit_message>
etiquetas de palet de AMI dentro de los excels de etiquetas de caja
Una hoja mas por destinacion (CHINA/JAPAN/FRANCE), dos etiquetas por A4.
El rango de cajas se lee de las cajas y no del rango del JSON, que se
queda viejo si se corrige un palet en la revision. Si a una sola caja le
falta el palet, esa destinacion va sin hoja y con aviso.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Etiquetas cajas/ETIQUETA CAJA AMI.xlsx
+++ b/docs/Etiquetas cajas/ETIQUETA CAJA AMI.xlsx
@@ -8,17 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jordi\Documents\Workspace\Packing List Automation\docs\Etiquetas cajas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE2F7A4-F485-4C89-BE47-6410CB2DE7EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18BF3FA6-0560-44FB-82D5-09F339FA9DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AMI CHINA" sheetId="1" r:id="rId1"/>
     <sheet name="AMI JAPAN" sheetId="2" r:id="rId2"/>
     <sheet name="AMI FRANCE" sheetId="3" r:id="rId3"/>
+    <sheet name="Etiquetas Palets JAPAN" sheetId="9" r:id="rId4"/>
+    <sheet name="Etiquetas Palets CHINA" sheetId="10" r:id="rId5"/>
+    <sheet name="Etiquetas Palets FRANCE" sheetId="11" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'AMI FRANCE'!$A$1:$D$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Etiquetas Palets CHINA'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Etiquetas Palets FRANCE'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Etiquetas Palets JAPAN'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -33,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="55">
   <si>
     <t>DHL GLOBAL FORWARDING CO.LTD</t>
   </si>
@@ -294,6 +300,131 @@
   <si>
     <t>14 / 84</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DESTINATAIRE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Consignee)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Nombre total de colis sur la palette
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Total number of packages on the palette)</t>
+    </r>
+  </si>
+  <si>
+    <t>64,58 Kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C/O AMI	
+N°305 HUTING RD	
+SONG JIANG DISTRICT	
+201616 SHANGHAI
+CHINA	</t>
+  </si>
+  <si>
+    <t>Nº 1 à Nº 12</t>
+  </si>
+  <si>
+    <t>FRANCE</t>
+  </si>
+  <si>
+    <t>AMI PARIS JAPAN
+MARUNI BUSINESS
+LOGISTICS CORPORATION - IBL PLAZA
+5-13, Chidori-Cho, Ichikawa-Shi
+272-0126 CHIBA - JAPAN</t>
+  </si>
+  <si>
+    <t>PUNTOTRES BAGS &amp; BELTS, S.L. C/INDUSTRIA 585-587 
+08918 BADALONA 
+SPAIN</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DESTINATION
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Destination)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">EXPEDITEUR
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Shipper / Sender)
+PROVENANCE
+(Origin)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Poids brut 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Black"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Total gross weight)</t>
+    </r>
+  </si>
+  <si>
+    <t>A.PARIS
+21 avenue Saint Mathurins
+60000 ALLONNE
+FRANCE</t>
+  </si>
+  <si>
+    <t>Nº 12 à Nº 24</t>
+  </si>
 </sst>
 </file>
 
@@ -302,11 +433,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="00000"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -472,8 +610,58 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -498,8 +686,14 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="27">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -809,207 +1003,262 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{1CA08267-AE73-40A6-8026-149D4D03D50B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1946,34 +2195,34 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="64"/>
+      <c r="C2" s="58"/>
     </row>
     <row r="3" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="62"/>
+      <c r="C3" s="60"/>
     </row>
     <row r="4" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="62"/>
+      <c r="C4" s="60"/>
     </row>
     <row r="5" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="62"/>
+      <c r="C5" s="60"/>
     </row>
     <row r="6" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="62"/>
+      <c r="C6" s="60"/>
     </row>
     <row r="7" spans="2:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
@@ -1991,19 +2240,19 @@
       <c r="B9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="59">
+      <c r="C9" s="63">
         <v>7703</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
-      <c r="C10" s="60"/>
+      <c r="C10" s="64"/>
     </row>
     <row r="11" spans="2:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="61" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2011,7 +2260,7 @@
       <c r="B12" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="58"/>
+      <c r="C12" s="62"/>
     </row>
     <row r="13" spans="2:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
@@ -2055,34 +2304,34 @@
       </c>
     </row>
     <row r="19" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="63" t="s">
+      <c r="B19" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C19" s="64"/>
+      <c r="C19" s="58"/>
     </row>
     <row r="20" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="62"/>
+      <c r="C20" s="60"/>
     </row>
     <row r="21" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="C21" s="62"/>
+      <c r="C21" s="60"/>
     </row>
     <row r="22" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="61" t="s">
+      <c r="B22" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="62"/>
+      <c r="C22" s="60"/>
     </row>
     <row r="23" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="62"/>
+      <c r="C23" s="60"/>
     </row>
     <row r="24" spans="2:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
@@ -2100,19 +2349,19 @@
       <c r="B26" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="59">
+      <c r="C26" s="63">
         <v>7703</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="6"/>
-      <c r="C27" s="60"/>
+      <c r="C27" s="64"/>
     </row>
     <row r="28" spans="2:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="57" t="s">
+      <c r="C28" s="61" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2120,7 +2369,7 @@
       <c r="B29" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="58"/>
+      <c r="C29" s="62"/>
     </row>
     <row r="30" spans="2:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
@@ -3130,11 +3379,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
     <mergeCell ref="C28:C29"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="C26:C27"/>
@@ -3144,6 +3388,11 @@
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.15748031496062992" bottom="0.15748031496062992" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
@@ -3164,26 +3413,26 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="64"/>
+      <c r="C2" s="58"/>
     </row>
     <row r="3" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="61"/>
-      <c r="C3" s="62"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="60"/>
     </row>
     <row r="4" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="62"/>
+      <c r="C4" s="60"/>
     </row>
     <row r="5" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="62"/>
+      <c r="C5" s="60"/>
     </row>
     <row r="6" spans="2:4" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
@@ -3201,13 +3450,13 @@
       <c r="B8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="59">
+      <c r="C8" s="63">
         <v>7697</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6"/>
-      <c r="C9" s="60"/>
+      <c r="C9" s="64"/>
     </row>
     <row r="10" spans="2:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
@@ -3268,26 +3517,26 @@
       <c r="B17" s="36"/>
     </row>
     <row r="18" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="63" t="s">
+      <c r="B18" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="64"/>
+      <c r="C18" s="58"/>
     </row>
     <row r="19" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="61"/>
-      <c r="C19" s="62"/>
+      <c r="B19" s="59"/>
+      <c r="C19" s="60"/>
     </row>
     <row r="20" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="62"/>
+      <c r="C20" s="60"/>
     </row>
     <row r="21" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="62"/>
+      <c r="C21" s="60"/>
     </row>
     <row r="22" spans="2:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
@@ -3305,13 +3554,13 @@
       <c r="B24" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="59">
+      <c r="C24" s="63">
         <v>7697</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="6"/>
-      <c r="C25" s="60"/>
+      <c r="C25" s="64"/>
     </row>
     <row r="26" spans="2:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
@@ -4337,11 +4586,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B18:C18"/>
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C8:C9"/>
@@ -4349,6 +4593,11 @@
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B18:C18"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" r:id="rId1"/>
@@ -7528,4 +7777,343 @@
   <pageSetup paperSize="9" scale="89" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B601899D-4438-4E83-A234-FFA0F93CF2B1}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
+  <dimension ref="B1:E14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.88671875" style="71" customWidth="1"/>
+    <col min="2" max="2" width="38.21875" style="71" customWidth="1"/>
+    <col min="3" max="3" width="44.21875" style="71" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" style="71" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="71"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E1" s="71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="82" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="80" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="74" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="80" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="74" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="76"/>
+    </row>
+    <row r="6" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="82" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="80" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="74" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="80" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="74" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="72" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="76"/>
+    </row>
+    <row r="13" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="73" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9128A729-64F1-48A2-8EAC-F3A5FD408861}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
+  <dimension ref="B1:E14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.88671875" style="71" customWidth="1"/>
+    <col min="2" max="2" width="38.21875" style="71" customWidth="1"/>
+    <col min="3" max="3" width="44.21875" style="71" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" style="71" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="71"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E1" s="71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="82" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="80" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="74" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="80" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="74" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="76"/>
+    </row>
+    <row r="6" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="82" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="80" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="74" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="80" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="74" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="72" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="76"/>
+    </row>
+    <row r="13" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="73" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C782E10-FDCF-4A17-B641-599E54C5B36C}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
+  <dimension ref="B1:E14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.88671875" style="71" customWidth="1"/>
+    <col min="2" max="2" width="38.21875" style="71" customWidth="1"/>
+    <col min="3" max="3" width="44.21875" style="71" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" style="71" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="71"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E1" s="71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="81" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="79" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="78" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="79" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="76"/>
+    </row>
+    <row r="6" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="77" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="2:5" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="81" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="79" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="81.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="78" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="79" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="72" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="76"/>
+    </row>
+    <row r="13" spans="2:5" ht="75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="73" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="37.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="77" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>